<commit_message>
ui table fix vol2
</commit_message>
<xml_diff>
--- a/data/tony/excel/802576637_2025_invoices.xlsx
+++ b/data/tony/excel/802576637_2025_invoices.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -629,6 +629,59 @@
       <c r="K4" t="inlineStr">
         <is>
           <t>9,4</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>400011600281002</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>800916954</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ΑΦΟΙ ΛΑΓΟΥ ΧΡΩΜΑΤΑ ΙΚΕ</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>TΔA</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>60939</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>10/11/2025</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Τιμολόγιο Πώλησης</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>33,06</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>7,93</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>40,99</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
διορθωση ui epsilon preview σε dark mode
</commit_message>
<xml_diff>
--- a/data/tony/excel/802576637_2025_invoices.xlsx
+++ b/data/tony/excel/802576637_2025_invoices.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -488,32 +488,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>400011615024455</t>
+          <t>400011823705209</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>800916954</t>
+          <t>800470153</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ΑΦΟΙ ΛΑΓΟΥ ΧΡΩΜΑΤΑ ΙΚΕ</t>
+          <t>GALAXY HELLAS ΕΜΠΟΡΙΚΗ – ΕΙΣΑΓΩΓΙΚΗ Ε.Ε.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>TΔA</t>
+          <t>ΤΔΑ</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>60984</t>
+          <t>4653</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>11/11/2025</t>
+          <t>01/12/2025</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -524,15 +524,68 @@
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
+          <t>24,06</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>5,77</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>29,83</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>400011615024455</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>800916954</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ΑΦΟΙ ΛΑΓΟΥ ΧΡΩΜΑΤΑ ΙΚΕ</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>TΔA</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>60984</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>11/11/2025</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Τιμολόγιο Πώλησης</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
           <t>104,99</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>23,91</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>128,90</t>
         </is>

</xml_diff>

<commit_message>
modal summary fix v2
</commit_message>
<xml_diff>
--- a/data/tony/excel/802576637_2025_invoices.xlsx
+++ b/data/tony/excel/802576637_2025_invoices.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -588,6 +588,210 @@
       <c r="K3" t="inlineStr">
         <is>
           <t>128,90</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>400011605611275</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>095736139</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ΕΜΠΗΛΕΧ ΜΟΝΟΠΡΟΣΩΠΗ ΕΠΕ ΗΛΕΚΤΡΟΛΟΓΙΚΩΝ ΕΙΔΩΝ</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>00ΤΔΓ</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>4885</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>10/11/2025</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Τιμολόγιο Πώλησης</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>82,27</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>19,74</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>102,01</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>400011830437904</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>094386010</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>PREMIER CAPITAL ΕΛΛΑΣ-ΔΙΑΧΕΙΡΙΣΗ ΚΑΙ ΛΕΙΤΟΥΡΓΙΑ ΕΣΤΙΑΤΟΡΙΩΝ ΜΟΝΟΠΡΟΣΩΠΗ ΑΝΩΝΥΜΗ ΕΤΑΙΡΕΙΑ</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>ΑΛΠ</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>165</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>25/09/2025</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>ΑΠΟΔΕΙΞΗ</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>9,4</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>9,4</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>400011622878368</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>094439854</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ΤΡΑΚΑΔΑΣ Α.Ε.</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>11Μ0ΤΔΑ</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>9480</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>12/11/2025</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Τιμολόγιο Πώλησης</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>69,29</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>16,63</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>85,92</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>400011830437905</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>094386010</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>PREMIER CAPITAL ΕΛΛΑΣ-ΔΙΑΧΕΙΡΙΣΗ ΚΑΙ ΛΕΙΤΟΥΡΓΙΑ ΕΣΤΙΑΤΟΡΙΩΝ ΜΟΝΟΠΡΟΣΩΠΗ ΑΝΩΝΥΜΗ ΕΤΑΙΡΕΙΑ</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>ΑΛΠ</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>165</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>25/09/2025</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>ΑΠΟΔΕΙΞΗ</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>9,4</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>9,4</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
modal summary  & repeat entry & reclassification fiixes
</commit_message>
<xml_diff>
--- a/data/tony/excel/802576637_2025_invoices.xlsx
+++ b/data/tony/excel/802576637_2025_invoices.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -647,149 +647,100 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>400011830437904</t>
+          <t>400011622878368</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>094386010</t>
+          <t>094439854</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>PREMIER CAPITAL ΕΛΛΑΣ-ΔΙΑΧΕΙΡΙΣΗ ΚΑΙ ΛΕΙΤΟΥΡΓΙΑ ΕΣΤΙΑΤΟΡΙΩΝ ΜΟΝΟΠΡΟΣΩΠΗ ΑΝΩΝΥΜΗ ΕΤΑΙΡΕΙΑ</t>
+          <t>ΤΡΑΚΑΔΑΣ Α.Ε.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>ΑΛΠ</t>
+          <t>11Μ0ΤΔΑ</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>165</t>
+          <t>9480</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>25/09/2025</t>
+          <t>12/11/2025</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>ΑΠΟΔΕΙΞΗ</t>
+          <t>Τιμολόγιο Πώλησης</t>
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>9,4</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr"/>
+          <t>69,29</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>16,63</t>
+        </is>
+      </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>9,4</t>
+          <t>85,92</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>400011622878368</t>
+          <t>400011830437904</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>094439854</t>
+          <t>094386010</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ΤΡΑΚΑΔΑΣ Α.Ε.</t>
+          <t>PREMIER CAPITAL ΕΛΛΑΣ-ΔΙΑΧΕΙΡΙΣΗ ΚΑΙ ΛΕΙΤΟΥΡΓΙΑ ΕΣΤΙΑΤΟΡΙΩΝ ΜΟΝΟΠΡΟΣΩΠΗ ΑΝΩΝΥΜΗ ΕΤΑΙΡΕΙΑ</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>11Μ0ΤΔΑ</t>
+          <t>ΑΛΠ</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>9480</t>
+          <t>165</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>12/11/2025</t>
+          <t>25/09/2025</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Τιμολόγιο Πώλησης</t>
+          <t>ΑΠΟΔΕΙΞΗ</t>
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>69,29</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>16,63</t>
-        </is>
-      </c>
+          <t>9,4</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
-        <is>
-          <t>85,92</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>400011830437905</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>094386010</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>PREMIER CAPITAL ΕΛΛΑΣ-ΔΙΑΧΕΙΡΙΣΗ ΚΑΙ ΛΕΙΤΟΥΡΓΙΑ ΕΣΤΙΑΤΟΡΙΩΝ ΜΟΝΟΠΡΟΣΩΠΗ ΑΝΩΝΥΜΗ ΕΤΑΙΡΕΙΑ</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>ΑΛΠ</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>165</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>25/09/2025</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>ΑΠΟΔΕΙΞΗ</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>9,4</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr">
         <is>
           <t>9,4</t>
         </is>

</xml_diff>